<commit_message>
Update GST collection revenues data
</commit_message>
<xml_diff>
--- a/data/gst_collection_revenues.xlsx
+++ b/data/gst_collection_revenues.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="4">
   <si>
     <t>period_date</t>
   </si>
@@ -32,7 +32,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <sz val="12.0"/>
       <color theme="1"/>
@@ -49,11 +49,6 @@
       <color theme="1"/>
       <name val="Aptos Narrow"/>
     </font>
-    <font>
-      <sz val="12.0"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -69,7 +64,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -77,9 +72,6 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="1" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -865,7 +857,7 @@
       </c>
     </row>
     <row r="52" ht="15.75" customHeight="1">
-      <c r="A52" s="4">
+      <c r="A52" s="2">
         <v>46082.0</v>
       </c>
       <c r="B52" s="1" t="s">
@@ -875,7 +867,17 @@
         <v>200064.0</v>
       </c>
     </row>
-    <row r="53" ht="15.75" customHeight="1"/>
+    <row r="53" ht="15.75" customHeight="1">
+      <c r="A53" s="2">
+        <v>46113.0</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C53" s="3">
+        <v>242702.0</v>
+      </c>
+    </row>
     <row r="54" ht="15.75" customHeight="1"/>
     <row r="55" ht="15.75" customHeight="1"/>
     <row r="56" ht="15.75" customHeight="1"/>

</xml_diff>